<commit_message>
Update Yousician dashboard v142
</commit_message>
<xml_diff>
--- a/Yousician Strategic Environment Database v3.9.xlsx
+++ b/Yousician Strategic Environment Database v3.9.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf99c2fe7082d414e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="Reafa9252017e4f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Players" sheetId="3" r:id="R5cbd6ebcdd414ac7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="One Pagers" sheetId="4" r:id="Ra835c7c685f34e8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Context" sheetId="5" r:id="R3587238bbf7547c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Moves" sheetId="6" r:id="Re99b43b8d8d640d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direct Learning Apps" sheetId="7" r:id="R1a07849da6914083"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="8" r:id="R7a8ef3652c364014"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Gaps" sheetId="9" r:id="Rb86638b06cfe4d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R55b7ecee5d3347ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="2" r:id="R7951d19e362c4d3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key Players" sheetId="3" r:id="Rb3cbd1f1fd3e4193"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="One Pagers" sheetId="4" r:id="R2117639c9bb8401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Internal Context" sheetId="5" r:id="R07519065427d462d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Market Moves" sheetId="6" r:id="R6f9c30c2729d44d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Direct Learning Apps" sheetId="7" r:id="Rf939af7064a748dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relationships" sheetId="8" r:id="R05797346bc2a4f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Gaps" sheetId="9" r:id="R515e351a51aa4477"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -164,12 +164,58 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="dk1"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="accent1"/>
-        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
+                <a:lumMod val="110000"/>
+                <a:satMod val="105000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
+                <a:lumMod val="105000"/>
+                <a:satMod val="109000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
+                <a:satMod val="103000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="50000">
+              <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
+                <a:satMod val="110000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
+                <a:lumMod val="99000"/>
+                <a:satMod val="120000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="5400000" scaled="0"/>
+        </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700">
@@ -282,7 +328,7 @@
         <x:v>Package rebuilt</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>2026-06-14</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -298,7 +344,7 @@
         <x:v>Key players</x:v>
       </x:c>
       <x:c r="B5" s="4" t="str">
-        <x:v>28</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -306,7 +352,7 @@
         <x:v>One-pager profiles</x:v>
       </x:c>
       <x:c r="B6" s="4" t="str">
-        <x:v>28</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -823,7 +869,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q4" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R4" s="11" t="str">
         <x:v>Learning product connected to one of the strongest guitar brands.</x:v>
@@ -909,7 +955,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q5" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R5" s="11" t="str">
         <x:v>Piano learning app focused on songs, guided lessons, and practice support.</x:v>
@@ -1081,7 +1127,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q7" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R7" s="11" t="str">
         <x:v>Influential guitar educator with a broad online learning footprint.</x:v>
@@ -1339,7 +1385,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q10" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R10" s="11" t="str">
         <x:v>Large music instrument and audio company with broad education relevance.</x:v>
@@ -1597,7 +1643,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q13" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R13" s="11" t="str">
         <x:v>Cloud music creation and collaboration ecosystem with strong creator and community signals.</x:v>
@@ -1855,7 +1901,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q16" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R16" s="11" t="str">
         <x:v>Sample, sound, and creator workflow platform.</x:v>
@@ -2027,7 +2073,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q18" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R18" s="11" t="str">
         <x:v>AI music generation platform that changes how non-musicians create complete songs.</x:v>
@@ -2113,7 +2159,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q19" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R19" s="11" t="str">
         <x:v>AI music generation platform for prompt-based song creation.</x:v>
@@ -2199,7 +2245,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q20" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R20" s="11" t="str">
         <x:v>AI-powered music practice and audio utility used by musicians and learners.</x:v>
@@ -2356,13 +2402,13 @@
         <x:v>SaaS, consumer, education</x:v>
       </x:c>
       <x:c r="L22" s="11" t="str">
-        <x:v>Private</x:v>
+        <x:v>Private; investor consortium led by Goldman Sachs Asset Management</x:v>
       </x:c>
       <x:c r="M22" s="11" t="str">
         <x:v>Research content generation and classroom AI</x:v>
       </x:c>
       <x:c r="N22" s="11" t="str">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="O22" s="11" t="str">
         <x:v>3</x:v>
@@ -2377,10 +2423,10 @@
         <x:v>Game-based learning platform with broad teacher and classroom reach.</x:v>
       </x:c>
       <x:c r="S22" s="11" t="str">
-        <x:v>Useful benchmark for learning engagement, classroom channels, and education buyers.</x:v>
+        <x:v>Useful benchmark for game based learning engagement, classroom channels, education buyers, and AI assisted content creation.</x:v>
       </x:c>
       <x:c r="T22" s="11" t="str">
-        <x:v>Public company/product sources linked; needs market validation</x:v>
+        <x:v>Official product and AI sources linked; ownership and market relevance should be cited before board use</x:v>
       </x:c>
       <x:c r="U22" s="11" t="str">
         <x:v>Low</x:v>
@@ -3317,7 +3363,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q33" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R33" s="11" t="str">
         <x:v>Long-running online guitar lesson platform with structured courses, songs, and learning tools.</x:v>
@@ -3489,7 +3535,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q35" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R35" s="11" t="str">
         <x:v>Modern guitar-learning platform built around structured pathways and contemporary player identity.</x:v>
@@ -3575,7 +3621,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q36" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R36" s="11" t="str">
         <x:v>Interactive music-learning service built around real instruments, song catalog, and feedback.</x:v>
@@ -3661,7 +3707,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q37" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R37" s="11" t="str">
         <x:v>Guitar-learning app connected to Gibson's hardware and brand ecosystem.</x:v>
@@ -3919,7 +3965,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q40" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R40" s="11" t="str">
         <x:v>Chord-recognition and play-along platform that turns songs into playable chord progressions.</x:v>
@@ -4177,7 +4223,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q43" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R43" s="11" t="str">
         <x:v>Default open platform for free music learning, creator-led lessons, discovery, and artist careers.</x:v>
@@ -4263,7 +4309,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q44" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R44" s="11" t="str">
         <x:v>Iconic guitar brand with a direct learning app and hardware-led beginner entry points.</x:v>
@@ -4349,7 +4395,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q45" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R45" s="11" t="str">
         <x:v>Smart guitar amp and app ecosystem connecting gear, tones, songs, and practice.</x:v>
@@ -4779,7 +4825,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q50" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R50" s="11" t="str">
         <x:v>Popular music production software known for fast beat-making and accessible creator workflows.</x:v>
@@ -5467,7 +5513,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q58" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R58" s="11" t="str">
         <x:v>AI audio platform expanding into full music generation from natural language prompts.</x:v>
@@ -5725,7 +5771,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q61" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R61" s="11" t="str">
         <x:v>Artist-facing platform for managing Spotify presence, audience insights, promotion, and artist business tools.</x:v>
@@ -5811,7 +5857,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="Q62" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R62" s="11" t="str">
         <x:v>Artist insight platform tied to TikTok's music discovery and fan engagement surface.</x:v>
@@ -5983,7 +6029,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="Q64" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R64" s="11" t="str">
         <x:v>Umbrella music education platform spanning drums, piano, guitar, singing, lessons, and community.</x:v>
@@ -6069,7 +6115,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="Q65" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R65" s="11" t="str">
         <x:v>Mobile guitar learning app focused on structured plans and guided practice.</x:v>
@@ -6327,7 +6373,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="Q68" s="11" t="str">
-        <x:v>TRUE</x:v>
+        <x:v>FALSE</x:v>
       </x:c>
       <x:c r="R68" s="11" t="str">
         <x:v>Mobile app that detects chords and song structure from audio to support self-guided playing.</x:v>
@@ -8867,7 +8913,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="21.110000610351562" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="13.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="21.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="21.110000610351562" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="21.110000610351562" hidden="0" customWidth="1"/>
@@ -8953,7 +8999,7 @@
         <x:v>https://apps.apple.com/us/developer/simply-ltd/id1019442026</x:v>
       </x:c>
       <x:c r="L2" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -8991,30 +9037,30 @@
         <x:v>https://www.musegroup.com/</x:v>
       </x:c>
       <x:c r="L3" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
+        <x:v>Teachers, schools and music education organizations / wider education</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>Fender Play</x:v>
+        <x:v>Duolingo</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>Learning product connected to one of the strongest guitar brands.</x:v>
+        <x:v>Consumer learning benchmark for habit formation, gamification, and subscription education.</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
+        <x:v>Very large public consumer education app</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
-        <x:v>Fender</x:v>
+        <x:v>Public company / Duolingo, Inc.</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
-        <x:v>Confirmed app feedback surface; broader AI/connected-instrument roadmap remains a monitoring hypothesis</x:v>
+        <x:v>AI personalization, tutoring, and content systems research target</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str">
-        <x:v>Shows how instrument makers can extend into software, subscriptions, and beginner journeys.</x:v>
+        <x:v>Not music-specific, but highly relevant for learning loops, retention, brand, and AI in education.</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
         <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
@@ -9026,33 +9072,33 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="K4" s="11" t="str">
-        <x:v>https://www.fender.com/play</x:v>
+        <x:v>https://investors.duolingo.com/</x:v>
       </x:c>
       <x:c r="L4" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
+        <x:v>Instrument brands, manufacturers and distributors</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Flowkey</x:v>
+        <x:v>Fender</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>Piano learning app focused on songs, guided lessons, and practice support.</x:v>
+        <x:v>Iconic guitar brand with reach across aspiration, hardware, education, and artist culture.</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>Established piano app</x:v>
+        <x:v>Major global brand</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
-        <x:v>flowkey GmbH; Yamaha partnership should be treated as partner context unless ownership is separately validated</x:v>
+        <x:v>Fender Musical Instruments Corporation / official company and product source; private ownership history not used as a main narrative claim.</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
-        <x:v>Confirmed feedback/product-learning surface; AI content generation remains a monitoring hypothesis</x:v>
+        <x:v>Research connected instrument and practice feedback initiatives</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str">
-        <x:v>Important benchmark for piano learning, catalog positioning, and conversion mechanics.</x:v>
+        <x:v>Instrument brands can shape the beginner funnel before users choose a learning app.</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
         <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
@@ -9061,925 +9107,13 @@
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="J5" s="11" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="K5" s="11" t="str">
-        <x:v>https://www.flowkey.com/en</x:v>
+        <x:v>https://www.fender.com/pages/about-fmic</x:v>
       </x:c>
       <x:c r="L5" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>JustinGuitar</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>Influential guitar educator with a broad online learning footprint.</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str">
-        <x:v>Large creator-led audience</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>JustinGuitar official learning site / creator-led educator platform; no ownership/investor claim used beyond public product identity.</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>Research how creator-led learning uses AI-assisted practice or content</x:v>
-      </x:c>
-      <x:c r="G6" s="11" t="str">
-        <x:v>Shows the power of trusted teachers and free content in shaping learner behavior.</x:v>
-      </x:c>
-      <x:c r="H6" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I6" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J6" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K6" s="11" t="str">
-        <x:v>https://www.justinguitar.com/</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>Fender</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="str">
-        <x:v>Iconic guitar brand with reach across aspiration, hardware, education, and artist culture.</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str">
-        <x:v>Major global brand</x:v>
-      </x:c>
-      <x:c r="E7" s="11" t="str">
-        <x:v>Fender Musical Instruments Corporation / official company and product source; private ownership history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="F7" s="11" t="str">
-        <x:v>Research connected instrument and practice feedback initiatives</x:v>
-      </x:c>
-      <x:c r="G7" s="11" t="str">
-        <x:v>Instrument brands can shape the beginner funnel before users choose a learning app.</x:v>
-      </x:c>
-      <x:c r="H7" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I7" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J7" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="K7" s="11" t="str">
-        <x:v>https://www.fender.com/pages/about-fmic</x:v>
-      </x:c>
-      <x:c r="L7" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="str">
-        <x:v>Yamaha</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="str">
-        <x:v>Large music instrument and audio company with broad education relevance.</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="str">
-        <x:v>Major global brand</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="str">
-        <x:v>Public company / Yamaha Corporation</x:v>
-      </x:c>
-      <x:c r="F8" s="11" t="str">
-        <x:v>Research smart instruments, learning integrations, and audio AI</x:v>
-      </x:c>
-      <x:c r="G8" s="11" t="str">
-        <x:v>Influences hardware access, music education channels, and partner possibilities.</x:v>
-      </x:c>
-      <x:c r="H8" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I8" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J8" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K8" s="11" t="str">
-        <x:v>https://www.yamaha.com/en/ir/</x:v>
-      </x:c>
-      <x:c r="L8" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="str">
-        <x:v>BandLab</x:v>
-      </x:c>
-      <x:c r="C9" s="11" t="str">
-        <x:v>Cloud music creation and collaboration ecosystem with strong creator and community signals.</x:v>
-      </x:c>
-      <x:c r="D9" s="11" t="str">
-        <x:v>Large creator community</x:v>
-      </x:c>
-      <x:c r="E9" s="11" t="str">
-        <x:v>BandLab Technologies / part of Caldecott Music Group; BandLab is the group flagship social music platform.</x:v>
-      </x:c>
-      <x:c r="F9" s="11" t="str">
-        <x:v>AI-assisted creation and creator workflow research target</x:v>
-      </x:c>
-      <x:c r="G9" s="11" t="str">
-        <x:v>Represents the shift from learning an instrument to making and sharing music quickly.</x:v>
-      </x:c>
-      <x:c r="H9" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I9" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J9" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="K9" s="11" t="str">
-        <x:v>https://bandlabtechnologies.com/</x:v>
-      </x:c>
-      <x:c r="L9" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="str">
-        <x:v>Splice</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="str">
-        <x:v>Sample, sound, and creator workflow platform.</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str">
-        <x:v>Large creator tool</x:v>
-      </x:c>
-      <x:c r="E10" s="11" t="str">
-        <x:v>Splice official music creation platform; private ownership/investor history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="str">
-        <x:v>AI search, generation, and workflow research target</x:v>
-      </x:c>
-      <x:c r="G10" s="11" t="str">
-        <x:v>Shows how hobbyists and creators pay for tools that accelerate making music.</x:v>
-      </x:c>
-      <x:c r="H10" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I10" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J10" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K10" s="11" t="str">
-        <x:v>https://splice.com/</x:v>
-      </x:c>
-      <x:c r="L10" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="B11" s="11" t="str">
-        <x:v>Suno</x:v>
-      </x:c>
-      <x:c r="C11" s="11" t="str">
-        <x:v>AI music generation platform that changes how non-musicians create complete songs.</x:v>
-      </x:c>
-      <x:c r="D11" s="11" t="str">
-        <x:v>High visibility AI platform</x:v>
-      </x:c>
-      <x:c r="E11" s="11" t="str">
-        <x:v>Suno official Series D source: over $400M raised at a $5.4B post-money valuation, led by Bond Capital with named investors.</x:v>
-      </x:c>
-      <x:c r="F11" s="11" t="str">
-        <x:v>Core AI music generation</x:v>
-      </x:c>
-      <x:c r="G11" s="11" t="str">
-        <x:v>May shift the meaning of music participation, motivation, and creation for casual users.</x:v>
-      </x:c>
-      <x:c r="H11" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I11" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J11" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="K11" s="11" t="str">
-        <x:v>https://suno.com/blog/series-d-announcement</x:v>
-      </x:c>
-      <x:c r="L11" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="B12" s="11" t="str">
-        <x:v>Udio</x:v>
-      </x:c>
-      <x:c r="C12" s="11" t="str">
-        <x:v>AI music generation platform for prompt-based song creation.</x:v>
-      </x:c>
-      <x:c r="D12" s="11" t="str">
-        <x:v>High visibility AI platform</x:v>
-      </x:c>
-      <x:c r="E12" s="11" t="str">
-        <x:v>Udio official/UMG source: AI music company backed by a16z, Redpoint, Hanwha, will.i.am, Steve Stoute, Kevin Wall and others.</x:v>
-      </x:c>
-      <x:c r="F12" s="11" t="str">
-        <x:v>Core AI music generation</x:v>
-      </x:c>
-      <x:c r="G12" s="11" t="str">
-        <x:v>Important to understand whether AI creation competes with, complements, or expands music learning.</x:v>
-      </x:c>
-      <x:c r="H12" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I12" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J12" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K12" s="11" t="str">
-        <x:v>https://www.universalmusic.com/universal-music-group-and-udio-announce-udios-first-strategic-agreements-for-new-licensed-ai-music-creation-platform/</x:v>
-      </x:c>
-      <x:c r="L12" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="B13" s="11" t="str">
-        <x:v>Moises</x:v>
-      </x:c>
-      <x:c r="C13" s="11" t="str">
-        <x:v>AI-powered music practice and audio utility used by musicians and learners.</x:v>
-      </x:c>
-      <x:c r="D13" s="11" t="str">
-        <x:v>Large musician utility</x:v>
-      </x:c>
-      <x:c r="E13" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="F13" s="11" t="str">
-        <x:v>Audio separation, practice tools, smart music utilities</x:v>
-      </x:c>
-      <x:c r="G13" s="11" t="str">
-        <x:v>Strong example of AI improving practice workflows without replacing instrument learning.</x:v>
-      </x:c>
-      <x:c r="H13" s="11" t="str">
-        <x:v>Needs app + company source</x:v>
-      </x:c>
-      <x:c r="I13" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J13" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="K13" s="11" t="str">
-        <x:v>https://moises.ai/</x:v>
-      </x:c>
-      <x:c r="L13" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="11" t="str">
-        <x:v>Teachers, schools and music education organizations / wider education</x:v>
-      </x:c>
-      <x:c r="B14" s="11" t="str">
-        <x:v>Duolingo</x:v>
-      </x:c>
-      <x:c r="C14" s="11" t="str">
-        <x:v>Consumer learning benchmark for habit formation, gamification, and subscription education.</x:v>
-      </x:c>
-      <x:c r="D14" s="11" t="str">
-        <x:v>Very large public consumer education app</x:v>
-      </x:c>
-      <x:c r="E14" s="11" t="str">
-        <x:v>Public company / Duolingo, Inc.</x:v>
-      </x:c>
-      <x:c r="F14" s="11" t="str">
-        <x:v>AI personalization, tutoring, and content systems research target</x:v>
-      </x:c>
-      <x:c r="G14" s="11" t="str">
-        <x:v>Not music-specific, but highly relevant for learning loops, retention, brand, and AI in education.</x:v>
-      </x:c>
-      <x:c r="H14" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I14" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J14" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K14" s="11" t="str">
-        <x:v>https://investors.duolingo.com/</x:v>
-      </x:c>
-      <x:c r="L14" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B15" s="11" t="str">
-        <x:v>Guitar Tricks</x:v>
-      </x:c>
-      <x:c r="C15" s="11" t="str">
-        <x:v>Long-running online guitar lesson platform with structured courses, songs, and learning tools.</x:v>
-      </x:c>
-      <x:c r="D15" s="11" t="str">
-        <x:v>Large online guitar education platform</x:v>
-      </x:c>
-      <x:c r="E15" s="11" t="str">
-        <x:v>Guitar Tricks Inc.</x:v>
-      </x:c>
-      <x:c r="F15" s="11" t="str">
-        <x:v>Research personalization, practice planning, and lesson recommendation signals</x:v>
-      </x:c>
-      <x:c r="G15" s="11" t="str">
-        <x:v>Important guitar-specific subscription benchmark for curriculum depth, song-led learning, and adult beginner messaging.</x:v>
-      </x:c>
-      <x:c r="H15" s="11" t="str">
-        <x:v>Public app/product sources linked; needs Appfigures + traffic data</x:v>
-      </x:c>
-      <x:c r="I15" s="11" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-      <x:c r="J15" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K15" s="11" t="str">
-        <x:v>https://www.guitartricks.com/</x:v>
-      </x:c>
-      <x:c r="L15" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B16" s="11" t="str">
-        <x:v>Pickup Music</x:v>
-      </x:c>
-      <x:c r="C16" s="11" t="str">
-        <x:v>Modern guitar-learning platform built around structured pathways and contemporary player identity.</x:v>
-      </x:c>
-      <x:c r="D16" s="11" t="str">
-        <x:v>Growing modern guitar platform</x:v>
-      </x:c>
-      <x:c r="E16" s="11" t="str">
-        <x:v>Pickup Music, Inc.</x:v>
-      </x:c>
-      <x:c r="F16" s="11" t="str">
-        <x:v>Research personalized feedback, pathway design, and practice accountability</x:v>
-      </x:c>
-      <x:c r="G16" s="11" t="str">
-        <x:v>Useful benchmark for higher-intent guitarists, modern aesthetics, community, and guided weekly practice.</x:v>
-      </x:c>
-      <x:c r="H16" s="11" t="str">
-        <x:v>Public product/app/company sources linked; needs traffic data</x:v>
-      </x:c>
-      <x:c r="I16" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J16" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K16" s="11" t="str">
-        <x:v>https://www.pickupmusic.com/</x:v>
-      </x:c>
-      <x:c r="L16" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B17" s="11" t="str">
-        <x:v>Rocksmith+</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="str">
-        <x:v>Interactive music-learning service built around real instruments, song catalog, and feedback.</x:v>
-      </x:c>
-      <x:c r="D17" s="11" t="str">
-        <x:v>Major game-backed learning brand</x:v>
-      </x:c>
-      <x:c r="E17" s="11" t="str">
-        <x:v>Ubisoft</x:v>
-      </x:c>
-      <x:c r="F17" s="11" t="str">
-        <x:v>Research note detection, adaptive difficulty, and song-based feedback mechanics</x:v>
-      </x:c>
-      <x:c r="G17" s="11" t="str">
-        <x:v>Important benchmark for real-time feedback, licensed songs, game-like practice, and multi-instrument expansion.</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I17" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J17" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K17" s="11" t="str">
-        <x:v>https://www.ubisoft.com/en-us/game/rocksmith/plus</x:v>
-      </x:c>
-      <x:c r="L17" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B18" s="11" t="str">
-        <x:v>Gibson App</x:v>
-      </x:c>
-      <x:c r="C18" s="11" t="str">
-        <x:v>Guitar-learning app connected to Gibson's hardware and brand ecosystem.</x:v>
-      </x:c>
-      <x:c r="D18" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
-      </x:c>
-      <x:c r="E18" s="11" t="str">
-        <x:v>Gibson App is visibly linked from Gibson official media/discover navigation and has its own official product site.</x:v>
-      </x:c>
-      <x:c r="F18" s="11" t="str">
-        <x:v>Research real-time feedback and brand-led personalization</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="str">
-        <x:v>Shows how a major guitar brand can bundle learning with instrument purchase and beginner motivation.</x:v>
-      </x:c>
-      <x:c r="H18" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I18" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J18" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K18" s="11" t="str">
-        <x:v>https://www.gibson.com/</x:v>
-      </x:c>
-      <x:c r="L18" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B19" s="11" t="str">
-        <x:v>Chordify</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="str">
-        <x:v>Chord-recognition and play-along platform that turns songs into playable chord progressions.</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="str">
-        <x:v>Large chord utility</x:v>
-      </x:c>
-      <x:c r="E19" s="11" t="str">
-        <x:v>Chordify official product/company identity; full ownership/investor history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="F19" s="11" t="str">
-        <x:v>Chord recognition, song parsing, and practice support</x:v>
-      </x:c>
-      <x:c r="G19" s="11" t="str">
-        <x:v>Owns a high-intent moment between song discovery and self-guided practice.</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I19" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J19" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K19" s="11" t="str">
-        <x:v>https://chordify.net/</x:v>
-      </x:c>
-      <x:c r="L19" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B20" s="11" t="str">
-        <x:v>YouTube</x:v>
-      </x:c>
-      <x:c r="C20" s="11" t="str">
-        <x:v>Default open platform for free music learning, creator-led lessons, discovery, and artist careers.</x:v>
-      </x:c>
-      <x:c r="D20" s="11" t="str">
-        <x:v>Massive global platform</x:v>
-      </x:c>
-      <x:c r="E20" s="11" t="str">
-        <x:v>YouTube for Artists official product surface; Google/Alphabet public-company context validated through Alphabet investor/SEC materials.</x:v>
-      </x:c>
-      <x:c r="F20" s="11" t="str">
-        <x:v>Recommendation, Shorts discovery, creator tools, and AI content policy</x:v>
-      </x:c>
-      <x:c r="G20" s="11" t="str">
-        <x:v>A major substitute and funnel for self-guided learning; it shapes inspiration, discovery, and expectations of free content.</x:v>
-      </x:c>
-      <x:c r="H20" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I20" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J20" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="K20" s="11" t="str">
-        <x:v>https://abc.xyz/investor/</x:v>
-      </x:c>
-      <x:c r="L20" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="B21" s="11" t="str">
-        <x:v>Gibson</x:v>
-      </x:c>
-      <x:c r="C21" s="11" t="str">
-        <x:v>Iconic guitar brand with a direct learning app and hardware-led beginner entry points.</x:v>
-      </x:c>
-      <x:c r="D21" s="11" t="str">
-        <x:v>Major guitar brand</x:v>
-      </x:c>
-      <x:c r="E21" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="F21" s="11" t="str">
-        <x:v>Research connected learning, app feedback, and brand-led beginner journeys</x:v>
-      </x:c>
-      <x:c r="G21" s="11" t="str">
-        <x:v>Hardware brands can capture learner intent before software choice and can bundle education into purchase moments.</x:v>
-      </x:c>
-      <x:c r="H21" s="11" t="str">
-        <x:v>Needs company + bundle performance source</x:v>
-      </x:c>
-      <x:c r="I21" s="11" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="J21" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K21" s="11" t="str">
-        <x:v>https://www.gibson.com/</x:v>
-      </x:c>
-      <x:c r="L21" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="B22" s="11" t="str">
-        <x:v>Positive Grid</x:v>
-      </x:c>
-      <x:c r="C22" s="11" t="str">
-        <x:v>Smart guitar amp and app ecosystem connecting gear, tones, songs, and practice.</x:v>
-      </x:c>
-      <x:c r="D22" s="11" t="str">
-        <x:v>Visible smart-amp ecosystem</x:v>
-      </x:c>
-      <x:c r="E22" s="11" t="str">
-        <x:v>Positive Grid Limited / official product company source.</x:v>
-      </x:c>
-      <x:c r="F22" s="11" t="str">
-        <x:v>AI tone generation, chord detection, smart practice, and connected hardware</x:v>
-      </x:c>
-      <x:c r="G22" s="11" t="str">
-        <x:v>Shows how hardware can become an app-led practice surface and compete for daily guitar time.</x:v>
-      </x:c>
-      <x:c r="H22" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I22" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J22" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K22" s="11" t="str">
-        <x:v>https://www.positivegrid.com/</x:v>
-      </x:c>
-      <x:c r="L22" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B23" s="11" t="str">
-        <x:v>FL Studio</x:v>
-      </x:c>
-      <x:c r="C23" s="11" t="str">
-        <x:v>Popular music production software known for fast beat-making and accessible creator workflows.</x:v>
-      </x:c>
-      <x:c r="D23" s="11" t="str">
-        <x:v>Major producer platform</x:v>
-      </x:c>
-      <x:c r="E23" s="11" t="str">
-        <x:v>Image-Line</x:v>
-      </x:c>
-      <x:c r="F23" s="11" t="str">
-        <x:v>Research browser DAW, AI-assisted production, and beginner creator onboarding</x:v>
-      </x:c>
-      <x:c r="G23" s="11" t="str">
-        <x:v>Shapes the path from musical interest to beat-making, production, and creator identity.</x:v>
-      </x:c>
-      <x:c r="H23" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I23" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J23" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K23" s="11" t="str">
-        <x:v>https://www.image-line.com/fl-studio/</x:v>
-      </x:c>
-      <x:c r="L23" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="B24" s="11" t="str">
-        <x:v>ElevenLabs Music</x:v>
-      </x:c>
-      <x:c r="C24" s="11" t="str">
-        <x:v>AI audio platform expanding into full music generation from natural language prompts.</x:v>
-      </x:c>
-      <x:c r="D24" s="11" t="str">
-        <x:v>High-profile AI audio company</x:v>
-      </x:c>
-      <x:c r="E24" s="11" t="str">
-        <x:v>ElevenLabs official company/product source includes AI music and creative-audio capabilities; private funding history requires separate validation.</x:v>
-      </x:c>
-      <x:c r="F24" s="11" t="str">
-        <x:v>Core AI music and audio generation</x:v>
-      </x:c>
-      <x:c r="G24" s="11" t="str">
-        <x:v>Important because major AI audio platforms may enter music creation, rights, and creator tooling at scale.</x:v>
-      </x:c>
-      <x:c r="H24" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I24" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J24" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K24" s="11" t="str">
-        <x:v>https://elevenlabs.io/</x:v>
-      </x:c>
-      <x:c r="L24" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="11" t="str">
-        <x:v>Investors, media, awards, funding and cultural drivers</x:v>
-      </x:c>
-      <x:c r="B25" s="11" t="str">
-        <x:v>Spotify for Artists</x:v>
-      </x:c>
-      <x:c r="C25" s="11" t="str">
-        <x:v>Artist-facing platform for managing Spotify presence, audience insights, promotion, and artist business tools.</x:v>
-      </x:c>
-      <x:c r="D25" s="11" t="str">
-        <x:v>Major global music platform</x:v>
-      </x:c>
-      <x:c r="E25" s="11" t="str">
-        <x:v>Spotify for Artists official product surface under Spotify.</x:v>
-      </x:c>
-      <x:c r="F25" s="11" t="str">
-        <x:v>Artist authenticity, AI music policy, recommendations, and creator tools</x:v>
-      </x:c>
-      <x:c r="G25" s="11" t="str">
-        <x:v>Important for how hobbyists understand music success, release goals, artist identity, and AI-authenticity debates.</x:v>
-      </x:c>
-      <x:c r="H25" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I25" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-      <x:c r="J25" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K25" s="11" t="str">
-        <x:v>https://artists.spotify.com/</x:v>
-      </x:c>
-      <x:c r="L25" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="11" t="str">
-        <x:v>Investors, media, awards, funding and cultural drivers</x:v>
-      </x:c>
-      <x:c r="B26" s="11" t="str">
-        <x:v>TikTok for Artists</x:v>
-      </x:c>
-      <x:c r="C26" s="11" t="str">
-        <x:v>Artist insight platform tied to TikTok's music discovery and fan engagement surface.</x:v>
-      </x:c>
-      <x:c r="D26" s="11" t="str">
-        <x:v>Massive short-form discovery platform</x:v>
-      </x:c>
-      <x:c r="E26" s="11" t="str">
-        <x:v>ByteDance</x:v>
-      </x:c>
-      <x:c r="F26" s="11" t="str">
-        <x:v>Recommendation, trend detection, creator tools, and AI content policy</x:v>
-      </x:c>
-      <x:c r="G26" s="11" t="str">
-        <x:v>TikTok can shape song discovery, cultural momentum, and what learners want to play.</x:v>
-      </x:c>
-      <x:c r="H26" s="11" t="str">
-        <x:v>Needs trend monitoring + music partnership source</x:v>
-      </x:c>
-      <x:c r="I26" s="11" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="J26" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K26" s="11" t="str">
-        <x:v>https://artists.tiktok.com/</x:v>
-      </x:c>
-      <x:c r="L26" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B27" s="11" t="str">
-        <x:v>Musora</x:v>
-      </x:c>
-      <x:c r="C27" s="11" t="str">
-        <x:v>Umbrella music education platform spanning drums, piano, guitar, singing, lessons, and community.</x:v>
-      </x:c>
-      <x:c r="D27" s="11" t="str">
-        <x:v>Large online music lesson ecosystem</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="F27" s="11" t="str">
-        <x:v>Research practice feedback, lesson recommendation, and cross-instrument learning paths</x:v>
-      </x:c>
-      <x:c r="G27" s="11" t="str">
-        <x:v>Adds an important multi-instrument subscription benchmark beyond single-instrument apps.</x:v>
-      </x:c>
-      <x:c r="H27" s="11" t="str">
-        <x:v>Needs app data + subscriber / traffic validation</x:v>
-      </x:c>
-      <x:c r="I27" s="11" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-      <x:c r="J27" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K27" s="11" t="str">
-        <x:v>https://www.musora.com/</x:v>
-      </x:c>
-      <x:c r="L27" s="11" t="str">
-        <x:v>2026-06-11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="B28" s="11" t="str">
-        <x:v>Fretello</x:v>
-      </x:c>
-      <x:c r="C28" s="11" t="str">
-        <x:v>Mobile guitar learning app focused on structured plans and guided practice.</x:v>
-      </x:c>
-      <x:c r="D28" s="11" t="str">
-        <x:v>Specialist guitar app</x:v>
-      </x:c>
-      <x:c r="E28" s="11" t="str">
-        <x:v>Fretello official specialist guitar-learning app; company/operator details require registry or app-store validation for legal precision.</x:v>
-      </x:c>
-      <x:c r="F28" s="11" t="str">
-        <x:v>Research personalization, adaptive plans, and feedback patterns</x:v>
-      </x:c>
-      <x:c r="G28" s="11" t="str">
-        <x:v>Directly relevant for guitar onboarding, lesson pacing, personalization, and app-store positioning.</x:v>
-      </x:c>
-      <x:c r="H28" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I28" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J28" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K28" s="11" t="str">
-        <x:v>https://fretello.com/app/</x:v>
-      </x:c>
-      <x:c r="L28" s="11" t="str">
-        <x:v>2026-06-13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="B29" s="11" t="str">
-        <x:v>Chord ai</x:v>
-      </x:c>
-      <x:c r="C29" s="11" t="str">
-        <x:v>Mobile app that detects chords and song structure from audio to support self-guided playing.</x:v>
-      </x:c>
-      <x:c r="D29" s="11" t="str">
-        <x:v>Visible AI practice utility</x:v>
-      </x:c>
-      <x:c r="E29" s="11" t="str">
-        <x:v>Chord ai official AI chord-recognition product; developer/legal entity should be validated from app-store or company records before precise ownership wording.</x:v>
-      </x:c>
-      <x:c r="F29" s="11" t="str">
-        <x:v>Core AI chord recognition and song parsing</x:v>
-      </x:c>
-      <x:c r="G29" s="11" t="str">
-        <x:v>Important because it moves AI directly into the song-to-practice moment that GuitarTuna/Yousician users care about.</x:v>
-      </x:c>
-      <x:c r="H29" s="11" t="str">
-        <x:v>Public source skim completed; credentialed performance or deeper investor history still pending where applicable.</x:v>
-      </x:c>
-      <x:c r="I29" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="J29" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-      <x:c r="K29" s="11" t="str">
-        <x:v>https://chordai.net/</x:v>
-      </x:c>
-      <x:c r="L29" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9991,16 +9125,16 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="17" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="13.890000343322754" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="28.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="28.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="28.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="28.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="28.889999389648438" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="28.889999389648438" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="23.219999313354492" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="28.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="28.889999389648438" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="28.889999389648438" hidden="0" customWidth="1"/>
@@ -10072,10 +9206,10 @@
         <x:v>Publicly visible consumer app; precise reach requires Appfigures or traffic validation.</x:v>
       </x:c>
       <x:c r="F2" s="11" t="str">
-        <x:v>Simply Guitar - Learn Guitar: 4.72 iOS public proxy, 383,142 iOS public proxy | Google Play public proxy: 10M+ downloads, 4.6 rating, 360K reviews. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures. | Simply Piano: 4.69 iOS public proxy, 824,845 iOS public proxy | Needs Appfigures; include as Simply portfolio app. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
+        <x:v>Simply Guitar - Learn Guitar: 4.72 iOS public proxy, 384,516 iOS public proxy | Google Play public proxy: 10M+ downloads, 4.6 rating, 360K reviews. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures. Apple public proxy: 4.72 rating, 384,516 ratings as of 2026-06-22. Google Play public proxy: 10M+ installs band as of 2026-06-22. Public proxy only, not Appfigures. | Simply Piano: 4.69 iOS public proxy, 827,951 iOS public proxy | Needs Appfigures; include as Simply portfolio app. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures. Apple public proxy: 4.69 rating, 827,951 ratings as of 2026-06-22. Google Play public proxy: 50M+ installs band as of 2026-06-22. Public proxy only, not Appfigures.</x:v>
       </x:c>
       <x:c r="G2" s="11" t="str">
-        <x:v>Simply Ltd / Simply app developer listing</x:v>
+        <x:v>Simply Ltd</x:v>
       </x:c>
       <x:c r="H2" s="11" t="str">
         <x:v>AI/personalization relevance should be validated before being treated as a product claim.</x:v>
@@ -10096,10 +9230,10 @@
         <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
       </x:c>
       <x:c r="N2" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
+        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
       </x:c>
       <x:c r="O2" s="11" t="str">
-        <x:v>Medium</x:v>
+        <x:v>Pending</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -10119,7 +9253,7 @@
         <x:v>Large global music community</x:v>
       </x:c>
       <x:c r="F3" s="11" t="str">
-        <x:v>Ultimate Guitar: Chords &amp; Tabs: 4.74 iOS public proxy, 459,471 iOS public proxy | Google Play public proxy: 10M+ downloads, 627K reviews. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
+        <x:v>Ultimate Guitar: Chords &amp; Tabs: 4.74 iOS public proxy, 461,398 iOS public proxy | Google Play public proxy: 10M+ downloads, 627K reviews. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures. Apple public proxy: 4.74 rating, 461,398 ratings as of 2026-06-22. Google Play public proxy: 10M+ installs band as of 2026-06-22. Public proxy only, not Appfigures.</x:v>
       </x:c>
       <x:c r="G3" s="11" t="str">
         <x:v>Muse Group</x:v>
@@ -10143,1232 +9277,104 @@
         <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
       </x:c>
       <x:c r="N3" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
+        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
       </x:c>
       <x:c r="O3" s="11" t="str">
-        <x:v>High</x:v>
+        <x:v>Low</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
-        <x:v>Fender Play</x:v>
+        <x:v>Duolingo</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
+        <x:v>Teachers, schools and music education organizations / wider education</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
+        <x:v>Consumer learning benchmark</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Learning product connected to one of the strongest guitar brands.</x:v>
+        <x:v>Consumer learning benchmark for habit formation, gamification, and subscription education.</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
+        <x:v>Very large public consumer education app</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
-        <x:v>Fender Play: Learn Guitar: 4.80 iOS public proxy, 60,626 iOS public proxy | Apple public proxy: 4.8 rating, 61K ratings; Google Play public proxy: 1M+ downloads, 13.2K reviews. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
+        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
       </x:c>
       <x:c r="G4" s="11" t="str">
-        <x:v>Fender</x:v>
+        <x:v>Public company</x:v>
       </x:c>
       <x:c r="H4" s="11" t="str">
-        <x:v>Confirmed app feedback surface; broader AI/connected-instrument roadmap remains a monitoring hypothesis</x:v>
+        <x:v>AI personalization and tutoring relevance should be validated before high-stakes use.</x:v>
       </x:c>
       <x:c r="I4" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
+        <x:v>2024-09-25: Duolingo Music was linked to a beginner-friendly portable piano product with Loog.</x:v>
       </x:c>
       <x:c r="J4" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
+        <x:v>Consumer learning benchmark</x:v>
       </x:c>
       <x:c r="K4" s="11" t="str">
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="L4" s="11" t="str">
-        <x:v>Shows how instrument makers can extend into software, subscriptions, and beginner journeys.</x:v>
+        <x:v>Not music-specific, but highly relevant for learning loops, retention, brand, and AI in education.</x:v>
       </x:c>
       <x:c r="M4" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
+        <x:v>No app-performance row mapped; add if app-based.</x:v>
       </x:c>
       <x:c r="N4" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
+        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
       </x:c>
       <x:c r="O4" s="11" t="str">
-        <x:v>High</x:v>
+        <x:v>Low</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
-        <x:v>Flowkey</x:v>
+        <x:v>Fender</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
+        <x:v>Instrument brands, manufacturers and distributors</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>Instrument learning app</x:v>
+        <x:v>Hardware ecosystem</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>Piano learning app focused on songs, guided lessons, and practice support.</x:v>
+        <x:v>Iconic guitar brand with reach across aspiration, hardware, education, and artist culture.</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
-        <x:v>Established piano app</x:v>
+        <x:v>Major global brand</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
-        <x:v>flowkey - Learn to Play Piano: 4.72 iOS public proxy, 63,813 iOS public proxy | Apple public proxy: 4.7 rating, 64K ratings; Google Play public proxy: 10M+ learners claim in listing. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
+        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
       </x:c>
       <x:c r="G5" s="11" t="str">
-        <x:v>flowkey GmbH; Yamaha partnership should be treated as partner context unless ownership is separately validated</x:v>
+        <x:v>Private</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
-        <x:v>Confirmed feedback/product-learning surface; AI content generation remains a monitoring hypothesis</x:v>
+        <x:v>Research connected instrument and practice feedback initiatives</x:v>
       </x:c>
       <x:c r="I5" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
+        <x:v>2026-06-10: Fender Studio Pro update was reported to integrate Moises stem separation and a smart studio assistant.</x:v>
       </x:c>
       <x:c r="J5" s="11" t="str">
-        <x:v>Instrument learning app</x:v>
+        <x:v>Hardware ecosystem</x:v>
       </x:c>
       <x:c r="K5" s="11" t="str">
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="L5" s="11" t="str">
-        <x:v>Important benchmark for piano learning, catalog positioning, and conversion mechanics.</x:v>
+        <x:v>Instrument brands can shape the beginner funnel before users choose a learning app.</x:v>
       </x:c>
       <x:c r="M5" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
+        <x:v>No app-performance row mapped; add if app-based.</x:v>
       </x:c>
       <x:c r="N5" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
+        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
       </x:c>
       <x:c r="O5" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="11" t="str">
-        <x:v>JustinGuitar</x:v>
-      </x:c>
-      <x:c r="B6" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C6" s="11" t="str">
-        <x:v>Creator-led practice ecosystem</x:v>
-      </x:c>
-      <x:c r="D6" s="11" t="str">
-        <x:v>Influential guitar educator with a broad online learning footprint.</x:v>
-      </x:c>
-      <x:c r="E6" s="11" t="str">
-        <x:v>Large creator-led audience</x:v>
-      </x:c>
-      <x:c r="F6" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G6" s="11" t="str">
-        <x:v>JustinGuitar official learning site / creator-led educator platform; no ownership/investor claim used beyond public product identity.</x:v>
-      </x:c>
-      <x:c r="H6" s="11" t="str">
-        <x:v>Research how creator-led learning uses AI-assisted practice or content</x:v>
-      </x:c>
-      <x:c r="I6" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J6" s="11" t="str">
-        <x:v>Creator-led practice ecosystem</x:v>
-      </x:c>
-      <x:c r="K6" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L6" s="11" t="str">
-        <x:v>Shows the power of trusted teachers and free content in shaping learner behavior.</x:v>
-      </x:c>
-      <x:c r="M6" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N6" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O6" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="11" t="str">
-        <x:v>Fender</x:v>
-      </x:c>
-      <x:c r="B7" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="C7" s="11" t="str">
-        <x:v>Hardware ecosystem</x:v>
-      </x:c>
-      <x:c r="D7" s="11" t="str">
-        <x:v>Iconic guitar brand with reach across aspiration, hardware, education, and artist culture.</x:v>
-      </x:c>
-      <x:c r="E7" s="11" t="str">
-        <x:v>Major global brand</x:v>
-      </x:c>
-      <x:c r="F7" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G7" s="11" t="str">
-        <x:v>Fender Musical Instruments Corporation / official company and product source; private ownership history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="H7" s="11" t="str">
-        <x:v>Research connected instrument and practice feedback initiatives</x:v>
-      </x:c>
-      <x:c r="I7" s="11" t="str">
-        <x:v>2026-06-10: Fender Studio Pro update was reported to integrate Moises stem separation and a smart studio assistant.</x:v>
-      </x:c>
-      <x:c r="J7" s="11" t="str">
-        <x:v>Hardware ecosystem</x:v>
-      </x:c>
-      <x:c r="K7" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L7" s="11" t="str">
-        <x:v>Instrument brands can shape the beginner funnel before users choose a learning app.</x:v>
-      </x:c>
-      <x:c r="M7" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N7" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O7" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="11" t="str">
-        <x:v>Yamaha</x:v>
-      </x:c>
-      <x:c r="B8" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="C8" s="11" t="str">
-        <x:v>Hardware and education ecosystem</x:v>
-      </x:c>
-      <x:c r="D8" s="11" t="str">
-        <x:v>Large music instrument and audio company with broad education relevance.</x:v>
-      </x:c>
-      <x:c r="E8" s="11" t="str">
-        <x:v>Major global brand</x:v>
-      </x:c>
-      <x:c r="F8" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G8" s="11" t="str">
-        <x:v>Public company / Yamaha Corporation</x:v>
-      </x:c>
-      <x:c r="H8" s="11" t="str">
-        <x:v>Research smart instruments, learning integrations, and audio AI</x:v>
-      </x:c>
-      <x:c r="I8" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J8" s="11" t="str">
-        <x:v>Hardware and education ecosystem</x:v>
-      </x:c>
-      <x:c r="K8" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L8" s="11" t="str">
-        <x:v>Influences hardware access, music education channels, and partner possibilities.</x:v>
-      </x:c>
-      <x:c r="M8" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N8" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O8" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="11" t="str">
-        <x:v>BandLab</x:v>
-      </x:c>
-      <x:c r="B9" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C9" s="11" t="str">
-        <x:v>Creation and social platform</x:v>
-      </x:c>
-      <x:c r="D9" s="11" t="str">
-        <x:v>Cloud music creation and collaboration ecosystem with strong creator and community signals.</x:v>
-      </x:c>
-      <x:c r="E9" s="11" t="str">
-        <x:v>Large creator community</x:v>
-      </x:c>
-      <x:c r="F9" s="11" t="str">
-        <x:v>BandLab Music Maker &amp; Beats: 4.75 iOS public proxy, 484,499 iOS public proxy | Apple public proxy: 4.8 rating, 484K ratings; company proxy: 100M+ creators and fans. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G9" s="11" t="str">
-        <x:v>BandLab Technologies / part of Caldecott Music Group; BandLab is the group flagship social music platform.</x:v>
-      </x:c>
-      <x:c r="H9" s="11" t="str">
-        <x:v>AI-assisted creation and creator-workflow relevance should be validated before high-stakes use.</x:v>
-      </x:c>
-      <x:c r="I9" s="11" t="str">
-        <x:v>2026-06-08: BandLab's help center updated SongStarter guidance for AI-generated song ideas. | 2025-02-01: BandLab continued to present itself as a 100M+ creator and fan platform.</x:v>
-      </x:c>
-      <x:c r="J9" s="11" t="str">
-        <x:v>Creation and social platform</x:v>
-      </x:c>
-      <x:c r="K9" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L9" s="11" t="str">
-        <x:v>Represents the shift from learning an instrument to making and sharing music quickly.</x:v>
-      </x:c>
-      <x:c r="M9" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N9" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O9" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="11" t="str">
-        <x:v>Splice</x:v>
-      </x:c>
-      <x:c r="B10" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C10" s="11" t="str">
-        <x:v>Creator marketplace</x:v>
-      </x:c>
-      <x:c r="D10" s="11" t="str">
-        <x:v>Sample, sound, and creator workflow platform.</x:v>
-      </x:c>
-      <x:c r="E10" s="11" t="str">
-        <x:v>Large creator tool</x:v>
-      </x:c>
-      <x:c r="F10" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G10" s="11" t="str">
-        <x:v>Splice official music creation platform; private ownership/investor history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="H10" s="11" t="str">
-        <x:v>AI search/generation/workflow relevance should be validated before high-stakes use.</x:v>
-      </x:c>
-      <x:c r="I10" s="11" t="str">
-        <x:v>2026-04-15: Splice announced generative AI tools tied to its creator compensation model. | 2025-10-02: Splice moved beyond samples with a cloud-connected instrument plugin drawing on Spitfire libraries. | 2025-04-28: Splice announced the acquisition of Spitfire Audio.</x:v>
-      </x:c>
-      <x:c r="J10" s="11" t="str">
-        <x:v>Creator marketplace</x:v>
-      </x:c>
-      <x:c r="K10" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L10" s="11" t="str">
-        <x:v>Shows how hobbyists and creators pay for tools that accelerate making music.</x:v>
-      </x:c>
-      <x:c r="M10" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N10" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O10" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" s="11" t="str">
-        <x:v>Suno</x:v>
-      </x:c>
-      <x:c r="B11" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="C11" s="11" t="str">
-        <x:v>AI creation disruptor</x:v>
-      </x:c>
-      <x:c r="D11" s="11" t="str">
-        <x:v>AI music generation platform that changes how non-musicians create complete songs.</x:v>
-      </x:c>
-      <x:c r="E11" s="11" t="str">
-        <x:v>High visibility AI platform</x:v>
-      </x:c>
-      <x:c r="F11" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G11" s="11" t="str">
-        <x:v>Suno official Series D source: over $400M raised at a $5.4B post-money valuation, led by Bond Capital with named investors.</x:v>
-      </x:c>
-      <x:c r="H11" s="11" t="str">
-        <x:v>Core AI music generation</x:v>
-      </x:c>
-      <x:c r="I11" s="11" t="str">
-        <x:v>June 3, 2026: Suno announced more than $400M in Series D funding at a $5.4B post-money valuation. 2026-01-22: Menlo framed Suno as participatory music creation in its Series C thesis. | 2025-11-25: Warner Music Group and Suno announced a partnership and settlement path for licensed AI models. | 2025-11-19: Suno raised a $250M Series C at a $2.45B post-money valuation.</x:v>
-      </x:c>
-      <x:c r="J11" s="11" t="str">
-        <x:v>AI creation disruptor</x:v>
-      </x:c>
-      <x:c r="K11" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L11" s="11" t="str">
-        <x:v>May shift the meaning of music participation, motivation, and creation for casual users.</x:v>
-      </x:c>
-      <x:c r="M11" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N11" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O11" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" s="11" t="str">
-        <x:v>Udio</x:v>
-      </x:c>
-      <x:c r="B12" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="C12" s="11" t="str">
-        <x:v>AI creation disruptor</x:v>
-      </x:c>
-      <x:c r="D12" s="11" t="str">
-        <x:v>AI music generation platform for prompt-based song creation.</x:v>
-      </x:c>
-      <x:c r="E12" s="11" t="str">
-        <x:v>High visibility AI platform</x:v>
-      </x:c>
-      <x:c r="F12" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G12" s="11" t="str">
-        <x:v>Udio official/UMG source: AI music company backed by a16z, Redpoint, Hanwha, will.i.am, Steve Stoute, Kevin Wall and others.</x:v>
-      </x:c>
-      <x:c r="H12" s="11" t="str">
-        <x:v>Core AI music generation</x:v>
-      </x:c>
-      <x:c r="I12" s="11" t="str">
-        <x:v>2026-06-10: Fender Studio Pro update was reported to integrate Moises stem separation and a smart studio assistant. | 2025-10-29: UMG and Udio settled litigation and announced agreements for a licensed AI music creation platform planned for 2026. | 2025-08-20: Moises launched AI Studio for adaptive AI music creation support.</x:v>
-      </x:c>
-      <x:c r="J12" s="11" t="str">
-        <x:v>AI creation disruptor</x:v>
-      </x:c>
-      <x:c r="K12" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L12" s="11" t="str">
-        <x:v>Important to understand whether AI creation competes with, complements, or expands music learning.</x:v>
-      </x:c>
-      <x:c r="M12" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N12" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O12" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="11" t="str">
-        <x:v>Moises</x:v>
-      </x:c>
-      <x:c r="B13" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="C13" s="11" t="str">
-        <x:v>AI practice utility</x:v>
-      </x:c>
-      <x:c r="D13" s="11" t="str">
-        <x:v>AI-powered music practice and audio utility used by musicians and learners.</x:v>
-      </x:c>
-      <x:c r="E13" s="11" t="str">
-        <x:v>Large musician utility</x:v>
-      </x:c>
-      <x:c r="F13" s="11" t="str">
-        <x:v>Moises: The Musician's App: 4.70 iOS public proxy, 26,579 iOS public proxy | Apple public proxy: 4.7 rating, 27K ratings; company / MBW proxy: Music.AI says Moises reached 50M users. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G13" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="H13" s="11" t="str">
-        <x:v>Audio separation, practice tools, smart music utilities</x:v>
-      </x:c>
-      <x:c r="I13" s="11" t="str">
-        <x:v>2026-06-10: Fender Studio Pro update was reported to integrate Moises stem separation and a smart studio assistant. | 2025-08-20: Moises launched AI Studio for adaptive AI music creation support. | 2025-01-22: Music.AI raised a $40M Series A and reported Moises at 50M users.</x:v>
-      </x:c>
-      <x:c r="J13" s="11" t="str">
-        <x:v>AI practice utility</x:v>
-      </x:c>
-      <x:c r="K13" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L13" s="11" t="str">
-        <x:v>Strong example of AI improving practice workflows without replacing instrument learning.</x:v>
-      </x:c>
-      <x:c r="M13" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N13" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O13" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" s="11" t="str">
-        <x:v>Duolingo</x:v>
-      </x:c>
-      <x:c r="B14" s="11" t="str">
-        <x:v>Teachers, schools and music education organizations / wider education</x:v>
-      </x:c>
-      <x:c r="C14" s="11" t="str">
-        <x:v>Consumer learning benchmark</x:v>
-      </x:c>
-      <x:c r="D14" s="11" t="str">
-        <x:v>Consumer learning benchmark for habit formation, gamification, and subscription education.</x:v>
-      </x:c>
-      <x:c r="E14" s="11" t="str">
-        <x:v>Very large public consumer education app</x:v>
-      </x:c>
-      <x:c r="F14" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G14" s="11" t="str">
-        <x:v>Public company / Duolingo, Inc.</x:v>
-      </x:c>
-      <x:c r="H14" s="11" t="str">
-        <x:v>AI personalization and tutoring relevance should be validated before high-stakes use.</x:v>
-      </x:c>
-      <x:c r="I14" s="11" t="str">
-        <x:v>2024-09-25: Duolingo Music was linked to a beginner-friendly portable piano product with Loog.</x:v>
-      </x:c>
-      <x:c r="J14" s="11" t="str">
-        <x:v>Consumer learning benchmark</x:v>
-      </x:c>
-      <x:c r="K14" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L14" s="11" t="str">
-        <x:v>Not music-specific, but highly relevant for learning loops, retention, brand, and AI in education.</x:v>
-      </x:c>
-      <x:c r="M14" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N14" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O14" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="11" t="str">
-        <x:v>Guitar Tricks</x:v>
-      </x:c>
-      <x:c r="B15" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C15" s="11" t="str">
-        <x:v>Structured guitar learning platform</x:v>
-      </x:c>
-      <x:c r="D15" s="11" t="str">
-        <x:v>Long-running online guitar lesson platform with structured courses, songs, and learning tools.</x:v>
-      </x:c>
-      <x:c r="E15" s="11" t="str">
-        <x:v>Large online guitar education platform</x:v>
-      </x:c>
-      <x:c r="F15" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G15" s="11" t="str">
-        <x:v>Guitar Tricks Inc.</x:v>
-      </x:c>
-      <x:c r="H15" s="11" t="str">
-        <x:v>Research personalization, practice planning, and lesson recommendation signals</x:v>
-      </x:c>
-      <x:c r="I15" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J15" s="11" t="str">
-        <x:v>Structured guitar learning platform</x:v>
-      </x:c>
-      <x:c r="K15" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L15" s="11" t="str">
-        <x:v>Important guitar-specific subscription benchmark for curriculum depth, song-led learning, and adult beginner messaging.</x:v>
-      </x:c>
-      <x:c r="M15" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N15" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O15" s="11" t="str">
-        <x:v>Pending</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="11" t="str">
-        <x:v>Pickup Music</x:v>
-      </x:c>
-      <x:c r="B16" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C16" s="11" t="str">
-        <x:v>Structured guitar learning platform</x:v>
-      </x:c>
-      <x:c r="D16" s="11" t="str">
-        <x:v>Modern guitar-learning platform built around structured pathways and contemporary player identity.</x:v>
-      </x:c>
-      <x:c r="E16" s="11" t="str">
-        <x:v>Growing modern guitar platform</x:v>
-      </x:c>
-      <x:c r="F16" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G16" s="11" t="str">
-        <x:v>Pickup Music, Inc.</x:v>
-      </x:c>
-      <x:c r="H16" s="11" t="str">
-        <x:v>Research personalized feedback, pathway design, and practice accountability</x:v>
-      </x:c>
-      <x:c r="I16" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J16" s="11" t="str">
-        <x:v>Structured guitar learning platform</x:v>
-      </x:c>
-      <x:c r="K16" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L16" s="11" t="str">
-        <x:v>Useful benchmark for higher-intent guitarists, modern aesthetics, community, and guided weekly practice.</x:v>
-      </x:c>
-      <x:c r="M16" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N16" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O16" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="11" t="str">
-        <x:v>Rocksmith+</x:v>
-      </x:c>
-      <x:c r="B17" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C17" s="11" t="str">
-        <x:v>Interactive song-learning service</x:v>
-      </x:c>
-      <x:c r="D17" s="11" t="str">
-        <x:v>Interactive music-learning service built around real instruments, song catalog, and feedback.</x:v>
-      </x:c>
-      <x:c r="E17" s="11" t="str">
-        <x:v>Major game-backed learning brand</x:v>
-      </x:c>
-      <x:c r="F17" s="11" t="str">
-        <x:v>Needs Appfigures plus Ubisoft platform data. Public proxy, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G17" s="11" t="str">
-        <x:v>Ubisoft</x:v>
-      </x:c>
-      <x:c r="H17" s="11" t="str">
-        <x:v>Research note detection, adaptive difficulty, and song-based feedback mechanics</x:v>
-      </x:c>
-      <x:c r="I17" s="11" t="str">
-        <x:v>2024-06-20: Rocksmith+ continued cross-platform subscription positioning for learning real songs with real instruments.</x:v>
-      </x:c>
-      <x:c r="J17" s="11" t="str">
-        <x:v>Interactive song-learning service</x:v>
-      </x:c>
-      <x:c r="K17" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L17" s="11" t="str">
-        <x:v>Important benchmark for real-time feedback, licensed songs, game-like practice, and multi-instrument expansion.</x:v>
-      </x:c>
-      <x:c r="M17" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N17" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O17" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="11" t="str">
-        <x:v>Gibson App</x:v>
-      </x:c>
-      <x:c r="B18" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C18" s="11" t="str">
-        <x:v>Brand-backed guitar learning app</x:v>
-      </x:c>
-      <x:c r="D18" s="11" t="str">
-        <x:v>Guitar-learning app connected to Gibson's hardware and brand ecosystem.</x:v>
-      </x:c>
-      <x:c r="E18" s="11" t="str">
-        <x:v>Brand-backed learning app</x:v>
-      </x:c>
-      <x:c r="F18" s="11" t="str">
-        <x:v>Needs Appfigures and public app-store validation. Public proxy, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="str">
-        <x:v>Gibson App is visibly linked from Gibson official media/discover navigation and has its own official product site.</x:v>
-      </x:c>
-      <x:c r="H18" s="11" t="str">
-        <x:v>Research real-time feedback and brand-led personalization</x:v>
-      </x:c>
-      <x:c r="I18" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J18" s="11" t="str">
-        <x:v>Brand-backed guitar learning app</x:v>
-      </x:c>
-      <x:c r="K18" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L18" s="11" t="str">
-        <x:v>Shows how a major guitar brand can bundle learning with instrument purchase and beginner motivation.</x:v>
-      </x:c>
-      <x:c r="M18" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N18" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O18" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="11" t="str">
-        <x:v>Chordify</x:v>
-      </x:c>
-      <x:c r="B19" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C19" s="11" t="str">
-        <x:v>Song-chord practice utility</x:v>
-      </x:c>
-      <x:c r="D19" s="11" t="str">
-        <x:v>Chord-recognition and play-along platform that turns songs into playable chord progressions.</x:v>
-      </x:c>
-      <x:c r="E19" s="11" t="str">
-        <x:v>Large chord utility</x:v>
-      </x:c>
-      <x:c r="F19" s="11" t="str">
-        <x:v>Needs Appfigures / public app-store validation. Public proxy, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G19" s="11" t="str">
-        <x:v>Chordify official product/company identity; full ownership/investor history not used as a main narrative claim.</x:v>
-      </x:c>
-      <x:c r="H19" s="11" t="str">
-        <x:v>Chord recognition, song parsing, and practice support</x:v>
-      </x:c>
-      <x:c r="I19" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J19" s="11" t="str">
-        <x:v>Song-chord practice utility</x:v>
-      </x:c>
-      <x:c r="K19" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L19" s="11" t="str">
-        <x:v>Owns a high-intent moment between song discovery and self-guided practice.</x:v>
-      </x:c>
-      <x:c r="M19" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N19" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O19" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="11" t="str">
-        <x:v>YouTube</x:v>
-      </x:c>
-      <x:c r="B20" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C20" s="11" t="str">
-        <x:v>Music discovery and creator platform</x:v>
-      </x:c>
-      <x:c r="D20" s="11" t="str">
-        <x:v>Default open platform for free music learning, creator-led lessons, discovery, and artist careers.</x:v>
-      </x:c>
-      <x:c r="E20" s="11" t="str">
-        <x:v>Massive global platform</x:v>
-      </x:c>
-      <x:c r="F20" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G20" s="11" t="str">
-        <x:v>YouTube for Artists official product surface; Google/Alphabet public-company context validated through Alphabet investor/SEC materials.</x:v>
-      </x:c>
-      <x:c r="H20" s="11" t="str">
-        <x:v>Recommendation, Shorts discovery, creator tools, and AI content policy</x:v>
-      </x:c>
-      <x:c r="I20" s="11" t="str">
-        <x:v>2026-06-10: Independent musicians sued Google over alleged use of YouTube-uploaded music for Lyria AI training. | 2026-04-30: Alphabet reported record quarterly growth for YouTube Music and Premium non-trial subscribers. | 2024-11-12: YouTube tested AI restyling of licensed songs for Shorts using Dream Track technology.</x:v>
-      </x:c>
-      <x:c r="J20" s="11" t="str">
-        <x:v>Music discovery and creator platform</x:v>
-      </x:c>
-      <x:c r="K20" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L20" s="11" t="str">
-        <x:v>A major substitute and funnel for self-guided learning; it shapes inspiration, discovery, and expectations of free content.</x:v>
-      </x:c>
-      <x:c r="M20" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N20" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O20" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="11" t="str">
-        <x:v>Gibson</x:v>
-      </x:c>
-      <x:c r="B21" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="C21" s="11" t="str">
-        <x:v>Hardware and brand ecosystem</x:v>
-      </x:c>
-      <x:c r="D21" s="11" t="str">
-        <x:v>Iconic guitar brand with a direct learning app and hardware-led beginner entry points.</x:v>
-      </x:c>
-      <x:c r="E21" s="11" t="str">
-        <x:v>Major guitar brand</x:v>
-      </x:c>
-      <x:c r="F21" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G21" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="H21" s="11" t="str">
-        <x:v>Research connected learning, app feedback, and brand-led beginner journeys</x:v>
-      </x:c>
-      <x:c r="I21" s="11" t="str">
-        <x:v>2026-05-22: Guitar media highlighted Rick Beato's live collaboration at Six-String Sanctuary and use of signature Gibson gear.</x:v>
-      </x:c>
-      <x:c r="J21" s="11" t="str">
-        <x:v>Hardware and brand ecosystem</x:v>
-      </x:c>
-      <x:c r="K21" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L21" s="11" t="str">
-        <x:v>Hardware brands can capture learner intent before software choice and can bundle education into purchase moments.</x:v>
-      </x:c>
-      <x:c r="M21" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N21" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O21" s="11" t="str">
         <x:v>Low</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="11" t="str">
-        <x:v>Positive Grid</x:v>
-      </x:c>
-      <x:c r="B22" s="11" t="str">
-        <x:v>Instrument brands, manufacturers and distributors</x:v>
-      </x:c>
-      <x:c r="C22" s="11" t="str">
-        <x:v>Smart amp and practice ecosystem</x:v>
-      </x:c>
-      <x:c r="D22" s="11" t="str">
-        <x:v>Smart guitar amp and app ecosystem connecting gear, tones, songs, and practice.</x:v>
-      </x:c>
-      <x:c r="E22" s="11" t="str">
-        <x:v>Visible smart-amp ecosystem</x:v>
-      </x:c>
-      <x:c r="F22" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G22" s="11" t="str">
-        <x:v>Positive Grid Limited / official product company source.</x:v>
-      </x:c>
-      <x:c r="H22" s="11" t="str">
-        <x:v>AI tone generation, chord detection, smart practice, and connected hardware</x:v>
-      </x:c>
-      <x:c r="I22" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J22" s="11" t="str">
-        <x:v>Smart amp and practice ecosystem</x:v>
-      </x:c>
-      <x:c r="K22" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L22" s="11" t="str">
-        <x:v>Shows how hardware can become an app-led practice surface and compete for daily guitar time.</x:v>
-      </x:c>
-      <x:c r="M22" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N22" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O22" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="11" t="str">
-        <x:v>FL Studio</x:v>
-      </x:c>
-      <x:c r="B23" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C23" s="11" t="str">
-        <x:v>Accessible production platform</x:v>
-      </x:c>
-      <x:c r="D23" s="11" t="str">
-        <x:v>Popular music production software known for fast beat-making and accessible creator workflows.</x:v>
-      </x:c>
-      <x:c r="E23" s="11" t="str">
-        <x:v>Major producer platform</x:v>
-      </x:c>
-      <x:c r="F23" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G23" s="11" t="str">
-        <x:v>Image-Line</x:v>
-      </x:c>
-      <x:c r="H23" s="11" t="str">
-        <x:v>Research browser DAW, AI-assisted production, and beginner creator onboarding</x:v>
-      </x:c>
-      <x:c r="I23" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J23" s="11" t="str">
-        <x:v>Accessible production platform</x:v>
-      </x:c>
-      <x:c r="K23" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L23" s="11" t="str">
-        <x:v>Shapes the path from musical interest to beat-making, production, and creator identity.</x:v>
-      </x:c>
-      <x:c r="M23" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N23" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O23" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="11" t="str">
-        <x:v>ElevenLabs Music</x:v>
-      </x:c>
-      <x:c r="B24" s="11" t="str">
-        <x:v>AI companies and AI initiatives</x:v>
-      </x:c>
-      <x:c r="C24" s="11" t="str">
-        <x:v>AI music and audio platform</x:v>
-      </x:c>
-      <x:c r="D24" s="11" t="str">
-        <x:v>AI audio platform expanding into full music generation from natural language prompts.</x:v>
-      </x:c>
-      <x:c r="E24" s="11" t="str">
-        <x:v>High-profile AI audio company</x:v>
-      </x:c>
-      <x:c r="F24" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G24" s="11" t="str">
-        <x:v>ElevenLabs official company/product source includes AI music and creative-audio capabilities; private funding history requires separate validation.</x:v>
-      </x:c>
-      <x:c r="H24" s="11" t="str">
-        <x:v>Core AI music and audio generation</x:v>
-      </x:c>
-      <x:c r="I24" s="11" t="str">
-        <x:v>2025-08-01: ElevenLabs launched Eleven Music for prompt-based music generation.</x:v>
-      </x:c>
-      <x:c r="J24" s="11" t="str">
-        <x:v>AI music and audio platform</x:v>
-      </x:c>
-      <x:c r="K24" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L24" s="11" t="str">
-        <x:v>Important because major AI audio platforms may enter music creation, rights, and creator tooling at scale.</x:v>
-      </x:c>
-      <x:c r="M24" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N24" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O24" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="11" t="str">
-        <x:v>Spotify for Artists</x:v>
-      </x:c>
-      <x:c r="B25" s="11" t="str">
-        <x:v>Investors, media, awards, funding and cultural drivers</x:v>
-      </x:c>
-      <x:c r="C25" s="11" t="str">
-        <x:v>Artist analytics and promotion platform</x:v>
-      </x:c>
-      <x:c r="D25" s="11" t="str">
-        <x:v>Artist-facing platform for managing Spotify presence, audience insights, promotion, and artist business tools.</x:v>
-      </x:c>
-      <x:c r="E25" s="11" t="str">
-        <x:v>Major global music platform</x:v>
-      </x:c>
-      <x:c r="F25" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G25" s="11" t="str">
-        <x:v>Spotify for Artists official product surface under Spotify.</x:v>
-      </x:c>
-      <x:c r="H25" s="11" t="str">
-        <x:v>Artist authenticity, AI music policy, recommendations, and creator tools</x:v>
-      </x:c>
-      <x:c r="I25" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J25" s="11" t="str">
-        <x:v>Artist analytics and promotion platform</x:v>
-      </x:c>
-      <x:c r="K25" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L25" s="11" t="str">
-        <x:v>Important for how hobbyists understand music success, release goals, artist identity, and AI-authenticity debates.</x:v>
-      </x:c>
-      <x:c r="M25" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N25" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O25" s="11" t="str">
-        <x:v>High</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="11" t="str">
-        <x:v>TikTok for Artists</x:v>
-      </x:c>
-      <x:c r="B26" s="11" t="str">
-        <x:v>Investors, media, awards, funding and cultural drivers</x:v>
-      </x:c>
-      <x:c r="C26" s="11" t="str">
-        <x:v>Music discovery and artist insights platform</x:v>
-      </x:c>
-      <x:c r="D26" s="11" t="str">
-        <x:v>Artist insight platform tied to TikTok's music discovery and fan engagement surface.</x:v>
-      </x:c>
-      <x:c r="E26" s="11" t="str">
-        <x:v>Massive short-form discovery platform</x:v>
-      </x:c>
-      <x:c r="F26" s="11" t="str">
-        <x:v>No public app-store proxy attached; use Appfigures or source validation before performance comparison.</x:v>
-      </x:c>
-      <x:c r="G26" s="11" t="str">
-        <x:v>ByteDance</x:v>
-      </x:c>
-      <x:c r="H26" s="11" t="str">
-        <x:v>Recommendation, trend detection, creator tools, and AI content policy</x:v>
-      </x:c>
-      <x:c r="I26" s="11" t="str">
-        <x:v>2025-06-03: TikTok for Artists launched globally after beta testing, initially in 26 countries. | 2025-04-10: Coverage indicated TikTok was preparing a dedicated artist insights platform before global launch.</x:v>
-      </x:c>
-      <x:c r="J26" s="11" t="str">
-        <x:v>Music discovery and artist insights platform</x:v>
-      </x:c>
-      <x:c r="K26" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L26" s="11" t="str">
-        <x:v>TikTok can shape song discovery, cultural momentum, and what learners want to play.</x:v>
-      </x:c>
-      <x:c r="M26" s="11" t="str">
-        <x:v>No app-performance row mapped; add if app-based.</x:v>
-      </x:c>
-      <x:c r="N26" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O26" s="11" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="11" t="str">
-        <x:v>Musora</x:v>
-      </x:c>
-      <x:c r="B27" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C27" s="11" t="str">
-        <x:v>Multi-instrument lesson ecosystem</x:v>
-      </x:c>
-      <x:c r="D27" s="11" t="str">
-        <x:v>Umbrella music education platform spanning drums, piano, guitar, singing, lessons, and community.</x:v>
-      </x:c>
-      <x:c r="E27" s="11" t="str">
-        <x:v>Large online music lesson ecosystem</x:v>
-      </x:c>
-      <x:c r="F27" s="11" t="str">
-        <x:v>Needs Appfigures plus web membership validation. Public proxy, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G27" s="11" t="str">
-        <x:v>Private</x:v>
-      </x:c>
-      <x:c r="H27" s="11" t="str">
-        <x:v>Research practice feedback, lesson recommendation, and cross-instrument learning paths</x:v>
-      </x:c>
-      <x:c r="I27" s="11" t="str">
-        <x:v>2025-09-01: Musora education brands continued to scale YouTube-led funnels for piano, drums, guitar and voice.</x:v>
-      </x:c>
-      <x:c r="J27" s="11" t="str">
-        <x:v>Multi-instrument lesson ecosystem</x:v>
-      </x:c>
-      <x:c r="K27" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L27" s="11" t="str">
-        <x:v>Adds an important multi-instrument subscription benchmark beyond single-instrument apps.</x:v>
-      </x:c>
-      <x:c r="M27" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N27" s="11" t="str">
-        <x:v>Validate Appfigures/traffic or investor data where applicable; confirm internal relationship owner.</x:v>
-      </x:c>
-      <x:c r="O27" s="11" t="str">
-        <x:v>Low</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="11" t="str">
-        <x:v>Fretello</x:v>
-      </x:c>
-      <x:c r="B28" s="11" t="str">
-        <x:v>Music learning apps and platforms</x:v>
-      </x:c>
-      <x:c r="C28" s="11" t="str">
-        <x:v>Guitar learning app</x:v>
-      </x:c>
-      <x:c r="D28" s="11" t="str">
-        <x:v>Mobile guitar learning app focused on structured plans and guided practice.</x:v>
-      </x:c>
-      <x:c r="E28" s="11" t="str">
-        <x:v>Specialist guitar app</x:v>
-      </x:c>
-      <x:c r="F28" s="11" t="str">
-        <x:v>Needs Appfigures; specialist guitar-learning app. Public proxy, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G28" s="11" t="str">
-        <x:v>Fretello official specialist guitar-learning app; company/operator details require registry or app-store validation for legal precision.</x:v>
-      </x:c>
-      <x:c r="H28" s="11" t="str">
-        <x:v>Research personalization, adaptive plans, and feedback patterns</x:v>
-      </x:c>
-      <x:c r="I28" s="11" t="str">
-        <x:v>No main-timeline recent-news item is used for this profile; source monitoring remains active.</x:v>
-      </x:c>
-      <x:c r="J28" s="11" t="str">
-        <x:v>Guitar learning app</x:v>
-      </x:c>
-      <x:c r="K28" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L28" s="11" t="str">
-        <x:v>Directly relevant for guitar onboarding, lesson pacing, personalization, and app-store positioning.</x:v>
-      </x:c>
-      <x:c r="M28" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N28" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O28" s="11" t="str">
-        <x:v>Medium</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="11" t="str">
-        <x:v>Chord ai</x:v>
-      </x:c>
-      <x:c r="B29" s="11" t="str">
-        <x:v>Music hobby software ecosystem</x:v>
-      </x:c>
-      <x:c r="C29" s="11" t="str">
-        <x:v>AI chord recognition app</x:v>
-      </x:c>
-      <x:c r="D29" s="11" t="str">
-        <x:v>Mobile app that detects chords and song structure from audio to support self-guided playing.</x:v>
-      </x:c>
-      <x:c r="E29" s="11" t="str">
-        <x:v>Visible AI practice utility</x:v>
-      </x:c>
-      <x:c r="F29" s="11" t="str">
-        <x:v>Chord ai: 4.65 iOS public proxy, 5,856 iOS public proxy | Needs Appfigures; public listings validate AI chord recognition. Public proxy, not Appfigures. iTunes Lookup refreshed 2026-06-11; public proxy only, not Appfigures.</x:v>
-      </x:c>
-      <x:c r="G29" s="11" t="str">
-        <x:v>Chord ai official AI chord-recognition product; developer/legal entity should be validated from app-store or company records before precise ownership wording.</x:v>
-      </x:c>
-      <x:c r="H29" s="11" t="str">
-        <x:v>Core AI chord recognition and song parsing</x:v>
-      </x:c>
-      <x:c r="I29" s="11" t="str">
-        <x:v>2024-07-15: Chord ai public listings positioned AI chord, beat and song-structure recognition as a play-any-song utility.</x:v>
-      </x:c>
-      <x:c r="J29" s="11" t="str">
-        <x:v>AI chord recognition app</x:v>
-      </x:c>
-      <x:c r="K29" s="11" t="str">
-        <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
-      </x:c>
-      <x:c r="L29" s="11" t="str">
-        <x:v>Important because it moves AI directly into the song-to-practice moment that GuitarTuna/Yousician users care about.</x:v>
-      </x:c>
-      <x:c r="M29" s="11" t="str">
-        <x:v>Credentialed Appfigures data is pending. Do not use this row for revenue, downloads, rank trend, review velocity, country mix or app-performance ranking.</x:v>
-      </x:c>
-      <x:c r="N29" s="11" t="str">
-        <x:v>Keep Appfigures/internal relationship validation separate; use paid database or direct source only for full investor/ownership history.</x:v>
-      </x:c>
-      <x:c r="O29" s="11" t="str">
-        <x:v>Medium</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -13347,7 +11353,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J2" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -13379,7 +11385,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J3" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -13411,7 +11417,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J4" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -13443,7 +11449,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J5" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -13475,7 +11481,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J6" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -13507,7 +11513,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J7" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -13539,7 +11545,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J8" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -13571,7 +11577,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J9" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -13603,7 +11609,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J10" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -13635,7 +11641,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J11" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -13665,7 +11671,7 @@
         <x:v>Internal relationship status not yet captured in this dataset. To be completed by Yousician.</x:v>
       </x:c>
       <x:c r="J12" s="11" t="str">
-        <x:v>2026-06-13</x:v>
+        <x:v>2026-06-22</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -14620,7 +12626,7 @@
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="E2" s="11" t="str">
-        <x:v>Export the Appfigures completion file and import the credentialed Appfigures export.</x:v>
+        <x:v>Export the Appfigures data request and run scripts/import_appfigures_export.py with --credentialed.</x:v>
       </x:c>
       <x:c r="F2" s="11" t="str">
         <x:v>Yousician / Appfigures credential owner</x:v>
@@ -14651,16 +12657,16 @@
         <x:v>Private company ownership and revenue</x:v>
       </x:c>
       <x:c r="B4" s="11" t="str">
-        <x:v>Mostly source-skimmed / paid database still required for deeper investor history and revenue</x:v>
+        <x:v>Partially validated / paid database or direct validation required</x:v>
       </x:c>
       <x:c r="C4" s="11" t="str">
-        <x:v>Public source skim now validates the remaining visible product/company identity and several parent-company or investor-context fields. Deep private-company ownership, investor history and revenue still require Crunchbase, PitchBook, Dealroom, registry or direct validation.</x:v>
+        <x:v>Public source status is captured, but ownership, investor history and revenue for private players require Crunchbase, PitchBook, Dealroom or direct validation.</x:v>
       </x:c>
       <x:c r="D4" s="11" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="E4" s="11" t="str">
-        <x:v>Use paid-database or direct company validation only if the next read needs detailed private ownership, investor history or revenue estimates.</x:v>
+        <x:v>Run a paid-database validation pass for private companies before investor/board usage.</x:v>
       </x:c>
       <x:c r="F4" s="11" t="str">
         <x:v>Research owner TBD</x:v>
@@ -14671,16 +12677,16 @@
         <x:v>Influencer multi-platform reach</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>Partially complete / YouTube source skim improved; platform exports still required</x:v>
+        <x:v>Partially complete / platform export required</x:v>
       </x:c>
       <x:c r="C5" s="11" t="str">
-        <x:v>YouTube public-profile/source proxies were refreshed for the previously open creator-reach rows. TikTok, Instagram and average views remain marked as pending platform export for campaign planning.</x:v>
+        <x:v>YouTube reach is included where visible. TikTok, Instagram and average views remain marked as pending platform export for campaign planning.</x:v>
       </x:c>
       <x:c r="D5" s="11" t="str">
-        <x:v>Medium</x:v>
+        <x:v>High</x:v>
       </x:c>
       <x:c r="E5" s="11" t="str">
-        <x:v>Use YouTube/TikTok/Instagram channel exports or creator tools to fill exact current reach and average-view fields before campaign use.</x:v>
+        <x:v>Use YouTube/TikTok/Instagram channel exports or creator tools to fill current reach and average-view fields.</x:v>
       </x:c>
       <x:c r="F5" s="11" t="str">
         <x:v>Creator/partnership owner TBD</x:v>

</xml_diff>